<commit_message>
Jagadeesh Changes till Oct-7-2025
</commit_message>
<xml_diff>
--- a/iPIM-Automation_JSONValidation/src/test/resources/excel/Test.xlsx
+++ b/iPIM-Automation_JSONValidation/src/test/resources/excel/Test.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jagadeesh.Reddy\Desktop\ipim\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jagadeesh.Reddy\Desktop\ipim\26sep\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AFAAE7-1099-44EA-862C-39736FE85BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B04F66-CE14-476A-AB55-761873A87CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="780" firstSheet="45" activeTab="48" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="780" firstSheet="45" activeTab="48" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddCatalogs" sheetId="80" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17822" uniqueCount="1978">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18026" uniqueCount="1985">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -6008,19 +6008,40 @@
     <t>verify_Prices_JSON_Verification_US</t>
   </si>
   <si>
+    <t>9870464</t>
+  </si>
+  <si>
+    <t>verify_Competitor_Price_JSON_Verification_US</t>
+  </si>
+  <si>
+    <t>Alternative item no. (selling, &lt;Public&gt;)</t>
+  </si>
+  <si>
+    <t>Competitor_ACESOUTH</t>
+  </si>
+  <si>
+    <t>verify_Product_Description_JSON_Verification_US</t>
+  </si>
+  <si>
+    <t>verify_Product_Media_JSON_Verification_US</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>5803732</t>
+  </si>
+  <si>
+    <t>verify_Web_Prices_JSON_Verification_US</t>
+  </si>
+  <si>
+    <t>verify_Divisional_Prices_JSON_Verification_US</t>
+  </si>
+  <si>
+    <t>verify_Product_Reference_JSON_Verification_US</t>
+  </si>
+  <si>
     <t>5803430</t>
-  </si>
-  <si>
-    <t>9870464</t>
-  </si>
-  <si>
-    <t>verify_Competitor_Price_JSON_Verification_US</t>
-  </si>
-  <si>
-    <t>Alternative item no. (selling, &lt;Public&gt;)</t>
-  </si>
-  <si>
-    <t>Competitor_ACESOUTH</t>
   </si>
 </sst>
 </file>
@@ -6133,7 +6154,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6218,6 +6239,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -6247,7 +6274,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
@@ -6378,6 +6405,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -52401,7 +52429,7 @@
 
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2F00-000000000000}">
-  <dimension ref="A1:AH9"/>
+  <dimension ref="A1:AH15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="52.21875" customWidth="1"/>
@@ -53058,7 +53086,7 @@
         <v>82</v>
       </c>
       <c r="G7" s="94" t="s">
-        <v>1973</v>
+        <v>1950</v>
       </c>
       <c r="H7" s="95" t="s">
         <v>24</v>
@@ -53248,7 +53276,7 @@
     </row>
     <row r="9" spans="1:34">
       <c r="A9" s="91" t="s">
-        <v>1975</v>
+        <v>1974</v>
       </c>
       <c r="B9" s="92" t="s">
         <v>106</v>
@@ -53266,7 +53294,7 @@
         <v>82</v>
       </c>
       <c r="G9" s="94" t="s">
-        <v>1974</v>
+        <v>1973</v>
       </c>
       <c r="H9" s="95" t="s">
         <v>24</v>
@@ -53338,16 +53366,640 @@
         <v>1752</v>
       </c>
       <c r="AE9" s="11" t="s">
-        <v>1976</v>
+        <v>1975</v>
       </c>
       <c r="AF9" s="11" t="s">
         <v>1969</v>
       </c>
       <c r="AG9" s="11" t="s">
+        <v>1975</v>
+      </c>
+      <c r="AH9" s="11" t="s">
         <v>1976</v>
       </c>
-      <c r="AH9" s="11" t="s">
+    </row>
+    <row r="10" spans="1:34">
+      <c r="A10" s="96" t="s">
         <v>1977</v>
+      </c>
+      <c r="B10" s="92" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="92" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="93" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G10" s="94" t="s">
+        <v>1950</v>
+      </c>
+      <c r="H10" s="95" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="93" t="s">
+        <v>349</v>
+      </c>
+      <c r="J10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="K10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="N10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="O10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="P10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q10" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="R10" s="93" t="s">
+        <v>1938</v>
+      </c>
+      <c r="S10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="T10" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="U10" s="93" t="s">
+        <v>1937</v>
+      </c>
+      <c r="V10" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="W10" s="93" t="s">
+        <v>1939</v>
+      </c>
+      <c r="X10" s="93" t="s">
+        <v>353</v>
+      </c>
+      <c r="Y10" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z10" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA10" s="93" t="s">
+        <v>1946</v>
+      </c>
+      <c r="AB10" s="93" t="s">
+        <v>1944</v>
+      </c>
+      <c r="AC10" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AD10" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AE10" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="AF10" s="11" t="s">
+        <v>1969</v>
+      </c>
+      <c r="AG10" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="AH10" s="11" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34">
+      <c r="A11" s="96" t="s">
+        <v>1978</v>
+      </c>
+      <c r="B11" s="92" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="92" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="93" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="94" t="s">
+        <v>1980</v>
+      </c>
+      <c r="H11" s="95" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="93" t="s">
+        <v>349</v>
+      </c>
+      <c r="J11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="K11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="N11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="O11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="P11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q11" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="R11" s="93" t="s">
+        <v>1938</v>
+      </c>
+      <c r="S11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="T11" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="U11" s="93" t="s">
+        <v>1937</v>
+      </c>
+      <c r="V11" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="W11" s="93" t="s">
+        <v>1939</v>
+      </c>
+      <c r="X11" s="93" t="s">
+        <v>353</v>
+      </c>
+      <c r="Y11" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z11" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA11" s="93" t="s">
+        <v>477</v>
+      </c>
+      <c r="AB11" s="93" t="s">
+        <v>1946</v>
+      </c>
+      <c r="AC11" s="93" t="s">
+        <v>1979</v>
+      </c>
+      <c r="AD11" s="93" t="s">
+        <v>1979</v>
+      </c>
+      <c r="AE11" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="AF11" s="11" t="s">
+        <v>1969</v>
+      </c>
+      <c r="AG11" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="AH11" s="11" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34">
+      <c r="A12" s="91" t="s">
+        <v>1981</v>
+      </c>
+      <c r="B12" s="92" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="92" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="93" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" s="94" t="s">
+        <v>1971</v>
+      </c>
+      <c r="H12" s="95" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" s="93" t="s">
+        <v>349</v>
+      </c>
+      <c r="J12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="N12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="O12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q12" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="R12" s="93" t="s">
+        <v>1938</v>
+      </c>
+      <c r="S12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="T12" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="U12" s="93" t="s">
+        <v>1937</v>
+      </c>
+      <c r="V12" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="W12" s="93" t="s">
+        <v>1939</v>
+      </c>
+      <c r="X12" s="93" t="s">
+        <v>353</v>
+      </c>
+      <c r="Y12" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z12" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA12" s="93" t="s">
+        <v>1944</v>
+      </c>
+      <c r="AB12" s="93" t="s">
+        <v>1944</v>
+      </c>
+      <c r="AC12" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AD12" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AE12" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AF12" s="11" t="s">
+        <v>1969</v>
+      </c>
+      <c r="AG12" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AH12" s="11" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34">
+      <c r="A13" s="91" t="s">
+        <v>1982</v>
+      </c>
+      <c r="B13" s="92" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="92" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" s="93" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G13" s="94" t="s">
+        <v>1971</v>
+      </c>
+      <c r="H13" s="95" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" s="93" t="s">
+        <v>349</v>
+      </c>
+      <c r="J13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="K13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="L13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="N13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="O13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="P13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q13" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="R13" s="93" t="s">
+        <v>1938</v>
+      </c>
+      <c r="S13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="U13" s="93" t="s">
+        <v>1937</v>
+      </c>
+      <c r="V13" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="W13" s="93" t="s">
+        <v>1939</v>
+      </c>
+      <c r="X13" s="93" t="s">
+        <v>353</v>
+      </c>
+      <c r="Y13" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z13" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA13" s="93" t="s">
+        <v>1944</v>
+      </c>
+      <c r="AB13" s="93" t="s">
+        <v>1944</v>
+      </c>
+      <c r="AC13" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AD13" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AE13" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AF13" s="11" t="s">
+        <v>1969</v>
+      </c>
+      <c r="AG13" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AH13" s="11" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34">
+      <c r="A14" s="91" t="s">
+        <v>1983</v>
+      </c>
+      <c r="B14" s="92" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="92" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="93" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="94" t="s">
+        <v>1984</v>
+      </c>
+      <c r="H14" s="95" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" s="93" t="s">
+        <v>349</v>
+      </c>
+      <c r="J14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="N14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="O14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="P14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q14" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="R14" s="93" t="s">
+        <v>1938</v>
+      </c>
+      <c r="S14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="T14" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="U14" s="93" t="s">
+        <v>1937</v>
+      </c>
+      <c r="V14" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="W14" s="93" t="s">
+        <v>1939</v>
+      </c>
+      <c r="X14" s="93" t="s">
+        <v>353</v>
+      </c>
+      <c r="Y14" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z14" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA14" s="93" t="s">
+        <v>681</v>
+      </c>
+      <c r="AB14" s="93" t="s">
+        <v>681</v>
+      </c>
+      <c r="AC14" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AD14" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AE14" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AF14" s="11" t="s">
+        <v>1969</v>
+      </c>
+      <c r="AG14" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AH14" s="11" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34">
+      <c r="A15" s="91" t="s">
+        <v>1983</v>
+      </c>
+      <c r="B15" s="92" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" s="92" t="s">
+        <v>107</v>
+      </c>
+      <c r="D15" s="93" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="G15" s="94" t="s">
+        <v>1980</v>
+      </c>
+      <c r="H15" s="95" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" s="93" t="s">
+        <v>349</v>
+      </c>
+      <c r="J15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="N15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="O15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q15" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="R15" s="93" t="s">
+        <v>1938</v>
+      </c>
+      <c r="S15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="T15" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="U15" s="93" t="s">
+        <v>1937</v>
+      </c>
+      <c r="V15" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="W15" s="93" t="s">
+        <v>1939</v>
+      </c>
+      <c r="X15" s="93" t="s">
+        <v>353</v>
+      </c>
+      <c r="Y15" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z15" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA15" s="93" t="s">
+        <v>681</v>
+      </c>
+      <c r="AB15" s="93" t="s">
+        <v>681</v>
+      </c>
+      <c r="AC15" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AD15" s="93" t="s">
+        <v>1752</v>
+      </c>
+      <c r="AE15" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AF15" s="11" t="s">
+        <v>1969</v>
+      </c>
+      <c r="AG15" s="11" t="s">
+        <v>1958</v>
+      </c>
+      <c r="AH15" s="11" t="s">
+        <v>1959</v>
       </c>
     </row>
   </sheetData>
@@ -53903,7 +54555,7 @@
       </c>
       <c r="N3" t="str">
         <f t="shared" ref="N3:N4" ca="1" si="0">CONCATENATE(E3," ",TEXT(TODAY(),"mm-dd-yyyy"))</f>
-        <v>SICA 09-16-2025</v>
+        <v>SICA 10-06-2025</v>
       </c>
       <c r="O3" t="s">
         <v>202</v>
@@ -54119,7 +54771,7 @@
       </c>
       <c r="N4" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>MICA 09-16-2025</v>
+        <v>MICA 10-06-2025</v>
       </c>
       <c r="O4" t="s">
         <v>202</v>
@@ -63115,6 +63767,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0af65dbd-c349-4f95-a569-a37e7dcda261">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a705add3-b55d-4a21-9da5-61558d9a88d9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004775ACE7CF61FD429C250F0EADD242CB" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bdc0ef193019ef7ec3c6044774d719fd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0af65dbd-c349-4f95-a569-a37e7dcda261" xmlns:ns3="a705add3-b55d-4a21-9da5-61558d9a88d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5eb62fd137b9132ea1ed680202856fff" ns2:_="" ns3:_="">
     <xsd:import namespace="0af65dbd-c349-4f95-a569-a37e7dcda261"/>
@@ -63369,27 +64041,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7BF3F34-769C-4AFA-8719-29B8EDC91EB1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0af65dbd-c349-4f95-a569-a37e7dcda261">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="a705add3-b55d-4a21-9da5-61558d9a88d9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B56E0B5-42C8-48C9-A658-2E92FF4B9C74}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0af65dbd-c349-4f95-a569-a37e7dcda261"/>
+    <ds:schemaRef ds:uri="a705add3-b55d-4a21-9da5-61558d9a88d9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2911B9E-6765-44F9-94CA-04166374824D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -63406,23 +64077,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7BF3F34-769C-4AFA-8719-29B8EDC91EB1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B56E0B5-42C8-48C9-A658-2E92FF4B9C74}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0af65dbd-c349-4f95-a569-a37e7dcda261"/>
-    <ds:schemaRef ds:uri="a705add3-b55d-4a21-9da5-61558d9a88d9"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>